<commit_message>
adde Old Timon character
</commit_message>
<xml_diff>
--- a/Game/db_tables/HallOfFame.xlsx
+++ b/Game/db_tables/HallOfFame.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="19">
   <si>
     <t>ID</t>
   </si>
@@ -26,6 +26,18 @@
     <t>Date</t>
   </si>
   <si>
+    <t>yosef3_1792876240470</t>
+  </si>
+  <si>
+    <t>yosef3</t>
+  </si>
+  <si>
+    <t>175</t>
+  </si>
+  <si>
+    <t>25/10/2026 00:10</t>
+  </si>
+  <si>
     <t>yosef 25/10/26_1792876098163</t>
   </si>
   <si>
@@ -47,16 +59,16 @@
     <t>10</t>
   </si>
   <si>
-    <t>yosef3_1792876240470</t>
-  </si>
-  <si>
-    <t>yosef3</t>
-  </si>
-  <si>
-    <t>175</t>
-  </si>
-  <si>
-    <t>25/10/2026 00:10</t>
+    <t>mike_1793074378062</t>
+  </si>
+  <si>
+    <t>mike</t>
+  </si>
+  <si>
+    <t>460</t>
+  </si>
+  <si>
+    <t>27/10/2026 06:12</t>
   </si>
 </sst>
 </file>
@@ -101,7 +113,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:CV4"/>
+  <dimension ref="A1:CV5"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -239,7 +251,7 @@
         <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="E3"/>
       <c r="F3"/>
@@ -340,16 +352,126 @@
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B4" t="s">
+        <v>13</v>
+      </c>
+      <c r="C4" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" t="s">
         <v>11</v>
       </c>
-      <c r="B4" t="s">
-        <v>12</v>
-      </c>
-      <c r="C4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D4" t="s">
-        <v>14</v>
+      <c r="E4"/>
+      <c r="F4"/>
+      <c r="G4"/>
+      <c r="H4"/>
+      <c r="I4"/>
+      <c r="J4"/>
+      <c r="K4"/>
+      <c r="L4"/>
+      <c r="M4"/>
+      <c r="N4"/>
+      <c r="O4"/>
+      <c r="P4"/>
+      <c r="Q4"/>
+      <c r="R4"/>
+      <c r="S4"/>
+      <c r="T4"/>
+      <c r="U4"/>
+      <c r="V4"/>
+      <c r="W4"/>
+      <c r="X4"/>
+      <c r="Y4"/>
+      <c r="Z4"/>
+      <c r="AA4"/>
+      <c r="AB4"/>
+      <c r="AC4"/>
+      <c r="AD4"/>
+      <c r="AE4"/>
+      <c r="AF4"/>
+      <c r="AG4"/>
+      <c r="AH4"/>
+      <c r="AI4"/>
+      <c r="AJ4"/>
+      <c r="AK4"/>
+      <c r="AL4"/>
+      <c r="AM4"/>
+      <c r="AN4"/>
+      <c r="AO4"/>
+      <c r="AP4"/>
+      <c r="AQ4"/>
+      <c r="AR4"/>
+      <c r="AS4"/>
+      <c r="AT4"/>
+      <c r="AU4"/>
+      <c r="AV4"/>
+      <c r="AW4"/>
+      <c r="AX4"/>
+      <c r="AY4"/>
+      <c r="AZ4"/>
+      <c r="BA4"/>
+      <c r="BB4"/>
+      <c r="BC4"/>
+      <c r="BD4"/>
+      <c r="BE4"/>
+      <c r="BF4"/>
+      <c r="BG4"/>
+      <c r="BH4"/>
+      <c r="BI4"/>
+      <c r="BJ4"/>
+      <c r="BK4"/>
+      <c r="BL4"/>
+      <c r="BM4"/>
+      <c r="BN4"/>
+      <c r="BO4"/>
+      <c r="BP4"/>
+      <c r="BQ4"/>
+      <c r="BR4"/>
+      <c r="BS4"/>
+      <c r="BT4"/>
+      <c r="BU4"/>
+      <c r="BV4"/>
+      <c r="BW4"/>
+      <c r="BX4"/>
+      <c r="BY4"/>
+      <c r="BZ4"/>
+      <c r="CA4"/>
+      <c r="CB4"/>
+      <c r="CC4"/>
+      <c r="CD4"/>
+      <c r="CE4"/>
+      <c r="CF4"/>
+      <c r="CG4"/>
+      <c r="CH4"/>
+      <c r="CI4"/>
+      <c r="CJ4"/>
+      <c r="CK4"/>
+      <c r="CL4"/>
+      <c r="CM4"/>
+      <c r="CN4"/>
+      <c r="CO4"/>
+      <c r="CP4"/>
+      <c r="CQ4"/>
+      <c r="CR4"/>
+      <c r="CS4"/>
+      <c r="CT4"/>
+      <c r="CU4"/>
+      <c r="CV4"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="s">
+        <v>15</v>
+      </c>
+      <c r="B5" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D5" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>